<commit_message>
Updated with headroom req
</commit_message>
<xml_diff>
--- a/RevitMappingData/ProjectClearanceRequirements.xlsx
+++ b/RevitMappingData/ProjectClearanceRequirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\source\repos\NewDigitalDelivery\DigitalDelivery\Resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ZAMORAMARIACARLOTAGA\Documents\GitHub\pocDataRepo\RevitMappingData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270496B2-8FD0-4303-A13C-BCE0A9EAECF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D27A045-1C11-48CF-BECB-6AFDB2B19A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12420" yWindow="-14940" windowWidth="30780" windowHeight="11235" xr2:uid="{D777F439-9358-4388-BAEA-A8A675FE2155}"/>
+    <workbookView xWindow="26445" yWindow="-14025" windowWidth="21510" windowHeight="11235" xr2:uid="{D777F439-9358-4388-BAEA-A8A675FE2155}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
   <si>
     <t>ItemKey</t>
   </si>
@@ -66,13 +66,19 @@
   </si>
   <si>
     <t>Ambulant</t>
+  </si>
+  <si>
+    <t>MOHH_Headroom</t>
+  </si>
+  <si>
+    <t>POC Standard_Headroom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -437,18 +443,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A7B1FA-DDB9-4761-BB99-B237A4A10C73}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -462,13 +469,19 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -482,13 +495,19 @@
         <v>0</v>
       </c>
       <c r="E2">
+        <v>2000</v>
+      </c>
+      <c r="F2">
         <v>1500</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>0</v>
       </c>
+      <c r="H2">
+        <v>2000</v>
+      </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -502,13 +521,19 @@
         <v>2000</v>
       </c>
       <c r="E3">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="F3">
         <v>1500</v>
       </c>
+      <c r="G3">
+        <v>1500</v>
+      </c>
+      <c r="H3">
+        <v>2000</v>
+      </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -522,10 +547,16 @@
         <v>0</v>
       </c>
       <c r="E4">
+        <v>2000</v>
+      </c>
+      <c r="F4">
         <v>1200</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>0</v>
+      </c>
+      <c r="H4">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>